<commit_message>
Recalibrated model for iMACC scenarios
</commit_message>
<xml_diff>
--- a/SubRES_TMPL/SubRES_TRA_NewVehicles.xlsx
+++ b/SubRES_TMPL/SubRES_TRA_NewVehicles.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rbsul\Documents\GitHub\times-ireland-model\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8DB867A-3B71-470A-99F5-9E94C8798621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6361C5-8AAF-4FD4-B5AD-D3A7E1FA45D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12643,18 +12643,14 @@
         <v>397.21899999999999</v>
       </c>
       <c r="J147" s="46">
-        <f t="shared" si="11"/>
-        <v>323.60950000000003</v>
+        <v>167.643</v>
       </c>
       <c r="K147" s="46">
-        <v>250</v>
-      </c>
-      <c r="L147" s="46">
-        <f t="shared" si="12"/>
-        <v>220</v>
-      </c>
+        <v>141.95599999999999</v>
+      </c>
+      <c r="L147" s="46"/>
       <c r="M147" s="46">
-        <v>130</v>
+        <v>113.565</v>
       </c>
       <c r="N147" s="46">
         <f>+N144*0.8</f>

</xml_diff>